<commit_message>
fix(importacoes): leitor de planilhas tipado e parser de data único (etapa 3, M05)
readSheet entrega a célula tipada: texto, número, máscara de zeros como
texto e data do Excel como data civil AAAA-MM-DD calculada do serial, sem
fuso; CSV é sempre texto. src/lib/importDate.ts é o parser único de datas
(container, Embarque de Vazios, programação, Granito, PIX, ZPT e Laden on
Board), com ano de quatro dígitos. Cabeçalho repetido ou duas colunas do
mesmo campo bloqueiam; linhas e abas ocultas são ignoradas com aviso no
seletor de arquivo; CSV Windows-1252 aceito com aviso; CE, CNPJ e CEP
numéricos com causa explícita (ADR 0078, item 22).

Os 9 it.fails de auditoriaLeituraPlanilhas viraram it, com checagens
novas de colunas duplicadas, linhas e abas ocultas e Windows-1252.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AFbzisLbhwnd9hRweKXeZ2
</commit_message>
<xml_diff>
--- a/public/templates/ce-mercante-modelo.xlsx
+++ b/public/templates/ce-mercante-modelo.xlsx
@@ -64,8 +64,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -121,10 +122,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -156,10 +157,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -411,7 +412,7 @@
       <c r="A2" t="str">
         <v>CSC456202060W00</v>
       </c>
-      <c r="B2" t="str">
+      <c r="B2" s="1" t="str">
         <v>123456789</v>
       </c>
     </row>
@@ -419,7 +420,7 @@
       <c r="A3" t="str">
         <v>CSC45620200300</v>
       </c>
-      <c r="B3" t="str">
+      <c r="B3" s="1" t="str">
         <v>987654321</v>
       </c>
     </row>

</xml_diff>

<commit_message>
B22 e B23: modelo de CE com 15 dígitos e exemplo de Nº de manifesto com 13
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EQMt4ftYPLMAD2mqQbsQTJ
</commit_message>
<xml_diff>
--- a/public/templates/ce-mercante-modelo.xlsx
+++ b/public/templates/ce-mercante-modelo.xlsx
@@ -1,52 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Modelo" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modelo" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -65,14 +42,81 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -397,36 +441,51 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
-        <v>BL</v>
-      </c>
-      <c r="B1" t="str">
-        <v>CE MERCANTE</v>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>BL</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>CE MERCANTE</t>
+        </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
-        <v>CSC456202060W00</v>
-      </c>
-      <c r="B2" s="1" t="str">
-        <v>123456789</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CSC456202060W00</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>122605051526081</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
-        <v>CSC45620200300</v>
-      </c>
-      <c r="B3" s="1" t="str">
-        <v>987654321</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CSC45620200300</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>122605051526082</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B3"/>
-  </ignoredErrors>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>